<commit_message>
[서버] ActorObject에 스탯값 얻기 멤버 추가, BasicStatComponent 추가, StatComponentBase 추가, CharacterStatComponent가 StatComponentBase 상속받게 수정, Monster 클래스 껍데기 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Monster.xlsx
+++ b/Development/Common/GameData/Monster.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Common\GameData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C16105-F50B-40F5-802E-51BD96B04BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65EC8864-3BE2-4314-A0F1-4FEF17CC0F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="90">
   <si>
     <t>데이터이름</t>
   </si>
@@ -161,18 +161,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>HP</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>all</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>int</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>server</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -284,51 +276,79 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>None</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>스탯</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>적용할스탯 타입</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>적용할스탯 값</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>AddHP</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>AddMP</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>AddAtk</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>참고이름</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>테스</t>
-  </si>
-  <si>
-    <t>Co</t>
-  </si>
-  <si>
-    <t>Di</t>
-  </si>
-  <si>
-    <t>Re</t>
-  </si>
-  <si>
-    <t>Sc</t>
+    <t>기본 스탯</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stat4</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatValue4</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stat5</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatValue5</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stat6</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatValue6</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stat7</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatValue7</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stat8</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatValue8</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StrAdd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>IntAdd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MoveSpdAdd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>HpAdd</t>
+  </si>
+  <si>
+    <t>MpAdd</t>
+  </si>
+  <si>
+    <t>PDefAdd</t>
+  </si>
+  <si>
+    <t>MDefAdd</t>
+  </si>
+  <si>
+    <t>AtkSpdAdd</t>
   </si>
 </sst>
 </file>
@@ -791,7 +811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.25" style="12" customWidth="1"/>
@@ -799,21 +819,20 @@
     <col min="3" max="3" width="30.25" style="3" customWidth="1"/>
     <col min="4" max="4" width="26" style="3" customWidth="1"/>
     <col min="5" max="5" width="23.625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.25" style="3" customWidth="1"/>
-    <col min="7" max="7" width="18.75" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="17.5" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.75" style="3" customWidth="1"/>
-    <col min="11" max="11" width="20.875" style="3" customWidth="1"/>
-    <col min="12" max="13" width="15.625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="13.25" style="3" customWidth="1"/>
-    <col min="15" max="15" width="16.375" style="3" customWidth="1"/>
-    <col min="16" max="16" width="15.625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="16.25" style="3" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="3"/>
+    <col min="6" max="6" width="18.75" style="3" customWidth="1"/>
+    <col min="7" max="7" width="13.375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17.5" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.75" style="3" customWidth="1"/>
+    <col min="10" max="10" width="20.875" style="3" customWidth="1"/>
+    <col min="11" max="12" width="15.625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="13.25" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.375" style="3" customWidth="1"/>
+    <col min="15" max="15" width="15.625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="16.25" style="3" customWidth="1"/>
+    <col min="17" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -821,7 +840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -838,29 +857,36 @@
         <v>38</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J2" s="4"/>
+        <v>43</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="K2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>73</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="L2" s="4"/>
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
     </row>
-    <row r="3" spans="1:17" s="7" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" s="7" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -870,40 +896,37 @@
       <c r="E3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6"/>
+      <c r="F3" s="6" t="s">
+        <v>45</v>
+      </c>
       <c r="G3" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>52</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="J3" s="6"/>
       <c r="K3" s="6"/>
-      <c r="L3" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -923,40 +946,67 @@
         <v>42</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="U4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="V4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="W4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="X4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -965,47 +1015,74 @@
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="Q5" s="8" t="s">
-        <v>64</v>
+        <v>54</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="S5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="T5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="U5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="V5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="W5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="X5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z5" s="8" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1017,24 +1094,43 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="J6" s="8" t="s">
+        <v>55</v>
+      </c>
       <c r="K6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q6" s="8"/>
+        <v>69</v>
+      </c>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z6" s="8"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1045,43 +1141,54 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8">
-        <v>100</v>
-      </c>
-      <c r="G7" s="8">
         <v>0</v>
       </c>
-      <c r="H7" s="8" t="b">
+      <c r="G7" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="I7" s="8">
+      <c r="H7" s="8">
         <v>0</v>
       </c>
-      <c r="J7" s="8" t="b">
+      <c r="I7" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="K7" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M7" s="8">
+      <c r="J7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8">
         <v>0</v>
       </c>
-      <c r="N7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="O7" s="8">
+      <c r="M7" s="8"/>
+      <c r="N7" s="8">
         <v>0</v>
       </c>
-      <c r="P7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="8">
+      <c r="O7" s="8"/>
+      <c r="P7" s="8">
         <v>0</v>
       </c>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8">
+        <v>0</v>
+      </c>
+      <c r="S7" s="8"/>
+      <c r="T7" s="8">
+        <v>0</v>
+      </c>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8">
+        <v>0</v>
+      </c>
+      <c r="W7" s="8"/>
+      <c r="X7" s="8">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="8"/>
+      <c r="Z7" s="8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:17" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>14</v>
       </c>
@@ -1089,7 +1196,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>39</v>
@@ -1098,43 +1205,70 @@
         <v>38</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>51</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="L8" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="P8" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="N8" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="O8" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="P8" s="10" t="s">
-        <v>67</v>
-      </c>
       <c r="Q8" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
+      </c>
+      <c r="R8" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="S8" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="T8" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="U8" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="V8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="W8" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="X8" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y8" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="Z8" s="10" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>50</v>
       </c>
@@ -1145,31 +1279,64 @@
         <v>16</v>
       </c>
       <c r="F9" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G9" s="3">
         <v>301</v>
       </c>
-      <c r="I9" s="3">
+      <c r="H9" s="3">
         <v>5.5</v>
       </c>
+      <c r="J9" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="K9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M9" s="3">
-        <v>100</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O9" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L9" s="3">
+        <v>10</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N9" s="3">
+        <v>10</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P9" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R9" s="3">
+        <v>100</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T9" s="3">
+        <v>100</v>
+      </c>
+      <c r="U9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V9" s="3">
+        <v>10</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X9" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z9" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>51</v>
       </c>
@@ -1180,31 +1347,64 @@
         <v>17</v>
       </c>
       <c r="F10" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G10" s="3">
         <v>21</v>
       </c>
-      <c r="I10" s="3">
+      <c r="H10" s="3">
         <v>6.6</v>
       </c>
+      <c r="J10" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="K10" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M10" s="3">
-        <v>200</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O10" s="3">
-        <v>200</v>
+        <v>82</v>
+      </c>
+      <c r="L10" s="3">
+        <v>10</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N10" s="3">
+        <v>10</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R10" s="3">
+        <v>100</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T10" s="3">
+        <v>100</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V10" s="3">
+        <v>10</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X10" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z10" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>52</v>
       </c>
@@ -1215,31 +1415,64 @@
         <v>18</v>
       </c>
       <c r="F11" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G11" s="3">
         <v>21</v>
       </c>
-      <c r="I11" s="3">
+      <c r="H11" s="3">
         <v>7.7</v>
       </c>
+      <c r="J11" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="K11" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M11" s="3">
-        <v>100</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O11" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L11" s="3">
+        <v>10</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N11" s="3">
+        <v>10</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P11" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R11" s="3">
+        <v>100</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T11" s="3">
+        <v>100</v>
+      </c>
+      <c r="U11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V11" s="3">
+        <v>10</v>
+      </c>
+      <c r="W11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X11" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y11" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z11" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>53</v>
       </c>
@@ -1250,30 +1483,63 @@
         <v>19</v>
       </c>
       <c r="F12" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G12" s="3">
         <v>21</v>
       </c>
-      <c r="I12" s="3">
+      <c r="H12" s="3">
         <v>8.8000000000000007</v>
       </c>
-      <c r="L12" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M12" s="3">
-        <v>100</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>100</v>
+      <c r="K12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L12" s="3">
+        <v>10</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N12" s="3">
+        <v>10</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P12" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R12" s="3">
+        <v>100</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T12" s="3">
+        <v>100</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V12" s="3">
+        <v>10</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X12" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z12" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B13" s="3">
         <v>54</v>
@@ -1285,31 +1551,64 @@
         <v>21</v>
       </c>
       <c r="F13" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G13" s="3">
         <v>21</v>
       </c>
-      <c r="H13" s="3" t="b">
+      <c r="G13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="I13" s="3">
+      <c r="H13" s="3">
         <v>9.9</v>
       </c>
-      <c r="L13" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M13" s="3">
-        <v>200</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q13" s="3">
-        <v>100</v>
+      <c r="K13" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L13" s="3">
+        <v>10</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N13" s="3">
+        <v>10</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P13" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R13" s="3">
+        <v>100</v>
+      </c>
+      <c r="S13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T13" s="3">
+        <v>100</v>
+      </c>
+      <c r="U13" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V13" s="3">
+        <v>10</v>
+      </c>
+      <c r="W13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X13" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y13" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z13" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>55</v>
       </c>
@@ -1320,31 +1619,64 @@
         <v>23</v>
       </c>
       <c r="F14" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G14" s="3">
         <v>201</v>
       </c>
-      <c r="I14" s="3">
+      <c r="H14" s="3">
         <v>11</v>
       </c>
+      <c r="J14" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="K14" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M14" s="3">
-        <v>100</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q14" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L14" s="3">
+        <v>10</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N14" s="3">
+        <v>10</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P14" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R14" s="3">
+        <v>100</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T14" s="3">
+        <v>100</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V14" s="3">
+        <v>10</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X14" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z14" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <v>56</v>
       </c>
@@ -1355,40 +1687,67 @@
         <v>25</v>
       </c>
       <c r="F15" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G15" s="3">
         <v>301</v>
       </c>
-      <c r="I15" s="3">
+      <c r="H15" s="3">
         <v>12.1</v>
       </c>
-      <c r="J15" s="3" t="b">
+      <c r="I15" s="3" t="b">
         <v>0</v>
       </c>
+      <c r="J15" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="K15" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M15" s="3">
-        <v>100</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O15" s="3">
-        <v>100</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q15" s="3">
-        <v>200</v>
+        <v>82</v>
+      </c>
+      <c r="L15" s="3">
+        <v>10</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N15" s="3">
+        <v>10</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P15" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R15" s="3">
+        <v>100</v>
+      </c>
+      <c r="S15" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T15" s="3">
+        <v>100</v>
+      </c>
+      <c r="U15" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V15" s="3">
+        <v>10</v>
+      </c>
+      <c r="W15" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X15" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y15" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z15" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>60</v>
       </c>
@@ -1399,40 +1758,67 @@
         <v>27</v>
       </c>
       <c r="F16" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G16" s="3">
         <v>301</v>
       </c>
-      <c r="I16" s="3">
+      <c r="H16" s="3">
         <v>13.2</v>
       </c>
-      <c r="J16" s="3" t="b">
+      <c r="I16" s="3" t="b">
         <v>0</v>
       </c>
+      <c r="J16" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="K16" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M16" s="3">
-        <v>200</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O16" s="3">
-        <v>200</v>
-      </c>
-      <c r="P16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L16" s="3">
+        <v>10</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N16" s="3">
+        <v>10</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P16" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R16" s="3">
+        <v>100</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T16" s="3">
+        <v>100</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V16" s="3">
+        <v>10</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X16" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z16" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <v>91</v>
       </c>
@@ -1443,31 +1829,64 @@
         <v>29</v>
       </c>
       <c r="F17" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G17" s="3">
         <v>99</v>
       </c>
-      <c r="I17" s="3">
+      <c r="H17" s="3">
         <v>14.3</v>
       </c>
+      <c r="J17" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="K17" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M17" s="3">
-        <v>100</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="O17" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L17" s="3">
+        <v>10</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N17" s="3">
+        <v>10</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P17" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R17" s="3">
+        <v>100</v>
+      </c>
+      <c r="S17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T17" s="3">
+        <v>100</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V17" s="3">
+        <v>10</v>
+      </c>
+      <c r="W17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X17" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y17" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z17" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <v>97</v>
       </c>
@@ -1478,25 +1897,64 @@
         <v>31</v>
       </c>
       <c r="F18" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G18" s="3">
         <v>99</v>
       </c>
-      <c r="I18" s="3">
+      <c r="H18" s="3">
         <v>15.4</v>
       </c>
+      <c r="J18" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="K18" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="M18" s="3">
-        <v>100</v>
+        <v>82</v>
+      </c>
+      <c r="L18" s="3">
+        <v>10</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N18" s="3">
+        <v>10</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P18" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R18" s="3">
+        <v>100</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T18" s="3">
+        <v>100</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V18" s="3">
+        <v>10</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X18" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z18" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <v>98</v>
       </c>
@@ -1507,19 +1965,64 @@
         <v>33</v>
       </c>
       <c r="F19" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G19" s="3">
         <v>99</v>
       </c>
-      <c r="I19" s="3">
+      <c r="H19" s="3">
         <v>16.5</v>
       </c>
+      <c r="J19" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="K19" s="3" t="s">
-        <v>63</v>
+        <v>82</v>
+      </c>
+      <c r="L19" s="3">
+        <v>10</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N19" s="3">
+        <v>10</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P19" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R19" s="3">
+        <v>100</v>
+      </c>
+      <c r="S19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T19" s="3">
+        <v>100</v>
+      </c>
+      <c r="U19" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V19" s="3">
+        <v>10</v>
+      </c>
+      <c r="W19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X19" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y19" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z19" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <v>99</v>
       </c>
@@ -1530,19 +2033,64 @@
         <v>33</v>
       </c>
       <c r="F20" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G20" s="3">
         <v>99</v>
       </c>
-      <c r="I20" s="3">
+      <c r="H20" s="3">
         <v>17.600000000000001</v>
       </c>
+      <c r="J20" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="K20" s="3" t="s">
-        <v>63</v>
+        <v>82</v>
+      </c>
+      <c r="L20" s="3">
+        <v>10</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N20" s="3">
+        <v>10</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P20" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R20" s="3">
+        <v>100</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T20" s="3">
+        <v>100</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V20" s="3">
+        <v>10</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X20" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z20" s="3">
+        <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
         <v>100</v>
       </c>
@@ -1553,16 +2101,61 @@
         <v>34</v>
       </c>
       <c r="F21" s="3">
-        <v>1000</v>
-      </c>
-      <c r="G21" s="3">
         <v>20</v>
       </c>
-      <c r="I21" s="3">
+      <c r="H21" s="3">
         <v>18.7</v>
       </c>
+      <c r="J21" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="K21" s="3" t="s">
-        <v>63</v>
+        <v>82</v>
+      </c>
+      <c r="L21" s="3">
+        <v>10</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N21" s="3">
+        <v>10</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P21" s="3">
+        <v>10</v>
+      </c>
+      <c r="Q21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R21" s="3">
+        <v>100</v>
+      </c>
+      <c r="S21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="T21" s="3">
+        <v>100</v>
+      </c>
+      <c r="U21" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="V21" s="3">
+        <v>10</v>
+      </c>
+      <c r="W21" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="X21" s="3">
+        <v>10</v>
+      </c>
+      <c r="Y21" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="Z21" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[데이터] Skill 데이터에 TelegraphPrefabPath, SfxLoop, SfxHitIgnoreMs 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Monster.xlsx
+++ b/Development/Common/GameData/Monster.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\MMOGameServerProject\Development\Common\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0DBE50-2F2F-4099-9025-AE36D6B3979B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637ADC47-D4BA-4A29-9A65-F09A9179EC26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38925" yWindow="6150" windowWidth="27045" windowHeight="14355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monster" sheetId="1" r:id="rId1"/>
@@ -1519,7 +1519,7 @@
         <v>61</v>
       </c>
       <c r="V9" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W9" s="3" t="s">
         <v>62</v>
@@ -1596,7 +1596,7 @@
         <v>61</v>
       </c>
       <c r="V10" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W10" s="3" t="s">
         <v>62</v>
@@ -1670,7 +1670,7 @@
         <v>61</v>
       </c>
       <c r="V11" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W11" s="3" t="s">
         <v>62</v>
@@ -1747,7 +1747,7 @@
         <v>61</v>
       </c>
       <c r="V12" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W12" s="3" t="s">
         <v>62</v>
@@ -1824,7 +1824,7 @@
         <v>61</v>
       </c>
       <c r="V13" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W13" s="3" t="s">
         <v>62</v>
@@ -1901,7 +1901,7 @@
         <v>61</v>
       </c>
       <c r="V14" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W14" s="3" t="s">
         <v>62</v>
@@ -1978,7 +1978,7 @@
         <v>61</v>
       </c>
       <c r="V15" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W15" s="3" t="s">
         <v>62</v>
@@ -2055,7 +2055,7 @@
         <v>61</v>
       </c>
       <c r="V16" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W16" s="3" t="s">
         <v>62</v>
@@ -2132,7 +2132,7 @@
         <v>61</v>
       </c>
       <c r="V17" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W17" s="3" t="s">
         <v>62</v>
@@ -2209,7 +2209,7 @@
         <v>61</v>
       </c>
       <c r="V18" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W18" s="3" t="s">
         <v>62</v>
@@ -2286,7 +2286,7 @@
         <v>61</v>
       </c>
       <c r="V19" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W19" s="3" t="s">
         <v>62</v>
@@ -2366,7 +2366,7 @@
         <v>61</v>
       </c>
       <c r="V20" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W20" s="3" t="s">
         <v>62</v>
@@ -2446,7 +2446,7 @@
         <v>61</v>
       </c>
       <c r="V21" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W21" s="3" t="s">
         <v>62</v>
@@ -2526,7 +2526,7 @@
         <v>61</v>
       </c>
       <c r="V22" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W22" s="3" t="s">
         <v>62</v>
@@ -2606,7 +2606,7 @@
         <v>61</v>
       </c>
       <c r="V23" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W23" s="3" t="s">
         <v>62</v>
@@ -2683,7 +2683,7 @@
         <v>61</v>
       </c>
       <c r="V24" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W24" s="3" t="s">
         <v>62</v>
@@ -2763,7 +2763,7 @@
         <v>61</v>
       </c>
       <c r="V25" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W25" s="3" t="s">
         <v>62</v>
@@ -2843,7 +2843,7 @@
         <v>61</v>
       </c>
       <c r="V26" s="3">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="W26" s="3" t="s">
         <v>62</v>

</xml_diff>